<commit_message>
if(timestep % 100 == 0)
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A26772EB-5B24-4A33-8EBD-34A7D28E2332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF0020E5-5661-4395-AEEC-C21AE4724229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -151,6 +151,10 @@
   </si>
   <si>
     <t>PIBT mainstream update 50</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PIBT mainstream update 100</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -476,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH5"/>
+  <dimension ref="A1:AH6"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" customWidth="1"/>
@@ -624,6 +628,17 @@
         <v>152</v>
       </c>
     </row>
+    <row r="6" spans="1:34" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6">
+        <v>5266</v>
+      </c>
+      <c r="D6">
+        <v>203</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
if(timestep % 20 == 0)
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0422955-FF0E-4443-BC9D-993F47BA5F64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F26E067D-4C00-40DB-AA4A-932F986105A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="29">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -131,6 +131,14 @@
   </si>
   <si>
     <t>比PIBT提升显著</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PIBT mainstream update 30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PIBT mainstream update 20</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -456,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X9"/>
+  <dimension ref="A1:X11"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" customWidth="1"/>
@@ -658,7 +666,7 @@
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
         <v>13</v>
@@ -673,18 +681,15 @@
         <v>1</v>
       </c>
       <c r="G8">
-        <v>4195</v>
+        <v>3713</v>
       </c>
       <c r="H8">
-        <v>152</v>
-      </c>
-      <c r="U8" t="s">
-        <v>19</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
         <v>13</v>
@@ -699,12 +704,61 @@
         <v>1</v>
       </c>
       <c r="G9">
+        <v>3852</v>
+      </c>
+      <c r="H9">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10">
+        <v>100</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>4195</v>
+      </c>
+      <c r="H10">
+        <v>152</v>
+      </c>
+      <c r="U10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11">
+        <v>100</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
         <v>5266</v>
       </c>
-      <c r="H9">
+      <c r="H11">
         <v>203</v>
       </c>
-      <c r="U9" t="s">
+      <c r="U11" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
if(timestep % 50 == 0)
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4254A52C-7DB4-42A1-8F3E-4B9BDEAB2B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96C184E3-E6DE-43F3-BE9E-69F94E760656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="36">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -146,11 +146,27 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>去掉居然没影响？</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>N/A</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>compare_addition update 20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>compare_addition update 30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>compare_addition update 50</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>融合后也没怎么变好</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>去掉没影响，可见不用担心任务饥饿的事情</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -476,7 +492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X12"/>
+  <dimension ref="A1:X15"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" customWidth="1"/>
@@ -619,7 +635,7 @@
         <v>73</v>
       </c>
       <c r="U4" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.3">
@@ -662,10 +678,10 @@
         <v>1</v>
       </c>
       <c r="G6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="U6" t="s">
         <v>26</v>
@@ -688,10 +704,10 @@
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="U7" t="s">
         <v>26</v>
@@ -714,10 +730,10 @@
         <v>2</v>
       </c>
       <c r="G8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.3">
@@ -816,6 +832,78 @@
       </c>
       <c r="U12" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E13">
+        <v>100</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>3781</v>
+      </c>
+      <c r="H13">
+        <v>75</v>
+      </c>
+      <c r="U13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14">
+        <v>100</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>3772</v>
+      </c>
+      <c r="H14">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15">
+        <v>100</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>3974</v>
+      </c>
+      <c r="H15">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
if(timestep % 10 == 0)
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{208EBD13-641F-41CB-82B7-DE726DACA2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3622D58A-9EFD-4A65-B584-3C0796BF5730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="36">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -98,10 +98,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>PIBT mainstream update 100</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>卧槽，更新时代精神并没有更好的效果</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -167,6 +163,10 @@
   </si>
   <si>
     <t>融合后也没怎么变好，可见elapse确实没什么所谓</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PIBT mainstream update 10</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -506,19 +506,19 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" t="s">
         <v>22</v>
-      </c>
-      <c r="E1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" t="s">
-        <v>23</v>
       </c>
       <c r="H1" t="s">
         <v>14</v>
@@ -574,7 +574,7 @@
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E2">
         <v>100</v>
@@ -597,7 +597,7 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E3">
         <v>150</v>
@@ -614,13 +614,13 @@
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E4">
         <v>100</v>
@@ -635,7 +635,7 @@
         <v>73</v>
       </c>
       <c r="U4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.3">
@@ -646,7 +646,7 @@
         <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E5">
         <v>100</v>
@@ -669,7 +669,7 @@
         <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E6">
         <v>100</v>
@@ -678,13 +678,13 @@
         <v>1</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="U6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.3">
@@ -695,7 +695,7 @@
         <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7">
         <v>150</v>
@@ -704,13 +704,13 @@
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="U7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.3">
@@ -721,7 +721,7 @@
         <v>13</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8">
         <v>150</v>
@@ -730,21 +730,21 @@
         <v>2</v>
       </c>
       <c r="G8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
         <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E9">
         <v>100</v>
@@ -753,10 +753,10 @@
         <v>1</v>
       </c>
       <c r="G9">
-        <v>3713</v>
+        <v>3761</v>
       </c>
       <c r="H9">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.3">
@@ -767,7 +767,7 @@
         <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E10">
         <v>100</v>
@@ -776,21 +776,21 @@
         <v>1</v>
       </c>
       <c r="G10">
-        <v>3852</v>
+        <v>3713</v>
       </c>
       <c r="H10">
-        <v>94</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="C11" t="s">
         <v>13</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E11">
         <v>100</v>
@@ -799,50 +799,47 @@
         <v>1</v>
       </c>
       <c r="G11">
-        <v>4195</v>
+        <v>3852</v>
       </c>
       <c r="H11">
-        <v>152</v>
-      </c>
-      <c r="U11" t="s">
-        <v>19</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12">
+        <v>100</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>4195</v>
+      </c>
+      <c r="H12">
+        <v>152</v>
+      </c>
+      <c r="U12" t="s">
         <v>18</v>
-      </c>
-      <c r="C12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12">
-        <v>100</v>
-      </c>
-      <c r="F12">
-        <v>1</v>
-      </c>
-      <c r="G12">
-        <v>5266</v>
-      </c>
-      <c r="H12">
-        <v>203</v>
-      </c>
-      <c r="U12" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
         <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E13">
         <v>100</v>
@@ -857,18 +854,18 @@
         <v>75</v>
       </c>
       <c r="U13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C14" t="s">
         <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E14">
         <v>100</v>
@@ -885,13 +882,13 @@
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C15" t="s">
         <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E15">
         <v>100</v>

</xml_diff>

<commit_message>
std::sort(A.begin(), A.end(), compare_region_cos); // 按优先级排序
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5801320-A7BD-4C2F-85F8-11122CC4DB2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0256D55-9213-4620-8D83-F78393B02322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="43">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1048,6 +1048,9 @@
       <c r="H20">
         <v>102</v>
       </c>
+      <c r="U20" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
@@ -1070,6 +1073,9 @@
       </c>
       <c r="H21">
         <v>102</v>
+      </c>
+      <c r="U21" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
std::sort(A.begin(), A.end(), compare); // 按优先级排序
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8DB5CC2-BEAE-4656-A215-BF743D0A0F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAF1A94B-3F20-4B24-9FDC-33D459AAD2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="51">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -211,6 +211,22 @@
   </si>
   <si>
     <t>region_cos比region_inner要好，但是不如PIBT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PIBT anti-mainstream update 50</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PIBT anti-mainstream update 30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PIBT anti-mainstream update 20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PIBT anti-mainstream update 10</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -536,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X24"/>
+  <dimension ref="A1:X28"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" customWidth="1"/>
@@ -877,7 +893,7 @@
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C13" t="s">
         <v>13</v>
@@ -891,19 +907,16 @@
       <c r="F13">
         <v>1</v>
       </c>
-      <c r="G13">
-        <v>3781</v>
-      </c>
-      <c r="H13">
-        <v>75</v>
-      </c>
-      <c r="U13" t="s">
-        <v>34</v>
+      <c r="G13" t="s">
+        <v>29</v>
+      </c>
+      <c r="H13" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="C14" t="s">
         <v>13</v>
@@ -917,16 +930,16 @@
       <c r="F14">
         <v>1</v>
       </c>
-      <c r="G14">
-        <v>3772</v>
-      </c>
-      <c r="H14">
-        <v>76</v>
+      <c r="G14" t="s">
+        <v>29</v>
+      </c>
+      <c r="H14" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="C15" t="s">
         <v>13</v>
@@ -940,16 +953,16 @@
       <c r="F15">
         <v>1</v>
       </c>
-      <c r="G15">
-        <v>3974</v>
-      </c>
-      <c r="H15">
-        <v>106</v>
+      <c r="G15" t="s">
+        <v>29</v>
+      </c>
+      <c r="H15" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
         <v>13</v>
@@ -972,7 +985,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
         <v>13</v>
@@ -987,15 +1000,18 @@
         <v>1</v>
       </c>
       <c r="G17">
-        <v>3632</v>
+        <v>3781</v>
       </c>
       <c r="H17">
-        <v>74</v>
+        <v>75</v>
+      </c>
+      <c r="U17" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C18" t="s">
         <v>13</v>
@@ -1010,15 +1026,15 @@
         <v>1</v>
       </c>
       <c r="G18">
-        <v>3877</v>
+        <v>3772</v>
       </c>
       <c r="H18">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C19" t="s">
         <v>13</v>
@@ -1033,18 +1049,15 @@
         <v>1</v>
       </c>
       <c r="G19">
-        <v>3741</v>
+        <v>3974</v>
       </c>
       <c r="H19">
-        <v>92</v>
-      </c>
-      <c r="U19" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C20" t="s">
         <v>13</v>
@@ -1058,19 +1071,16 @@
       <c r="F20">
         <v>1</v>
       </c>
-      <c r="G20">
-        <v>4008</v>
-      </c>
-      <c r="H20">
-        <v>102</v>
-      </c>
-      <c r="U20" t="s">
-        <v>42</v>
+      <c r="G20" t="s">
+        <v>29</v>
+      </c>
+      <c r="H20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C21" t="s">
         <v>13</v>
@@ -1085,18 +1095,15 @@
         <v>1</v>
       </c>
       <c r="G21">
-        <v>3748</v>
+        <v>3632</v>
       </c>
       <c r="H21">
-        <v>102</v>
-      </c>
-      <c r="U21" t="s">
-        <v>42</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C22" t="s">
         <v>13</v>
@@ -1111,18 +1118,15 @@
         <v>1</v>
       </c>
       <c r="G22">
-        <v>3592</v>
+        <v>3877</v>
       </c>
       <c r="H22">
-        <v>73</v>
-      </c>
-      <c r="U22" t="s">
-        <v>46</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C23" t="s">
         <v>13</v>
@@ -1137,38 +1141,142 @@
         <v>1</v>
       </c>
       <c r="G23">
-        <v>3679</v>
+        <v>3741</v>
       </c>
       <c r="H23">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="U23" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E24">
+        <v>100</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>4008</v>
+      </c>
+      <c r="H24">
+        <v>102</v>
+      </c>
+      <c r="U24" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>41</v>
+      </c>
+      <c r="C25" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25">
+        <v>100</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25">
+        <v>3748</v>
+      </c>
+      <c r="H25">
+        <v>102</v>
+      </c>
+      <c r="U25" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" t="s">
+        <v>20</v>
+      </c>
+      <c r="E26">
+        <v>100</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>3592</v>
+      </c>
+      <c r="H26">
+        <v>73</v>
+      </c>
+      <c r="U26" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27">
+        <v>100</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27">
+        <v>3679</v>
+      </c>
+      <c r="H27">
+        <v>75</v>
+      </c>
+      <c r="U27" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>45</v>
       </c>
-      <c r="C24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" t="s">
-        <v>20</v>
-      </c>
-      <c r="E24">
-        <v>100</v>
-      </c>
-      <c r="F24">
-        <v>1</v>
-      </c>
-      <c r="G24">
+      <c r="C28" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" t="s">
+        <v>20</v>
+      </c>
+      <c r="E28">
+        <v>100</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
         <v>3885</v>
       </c>
-      <c r="H24">
+      <c r="H28">
         <v>86</v>
       </c>
-      <c r="U24" t="s">
+      <c r="U28" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>

<commit_message>
std::sort(A.begin(), A.end(), compare_mainstream); // 按优先级排序
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF5874DF-3282-4BA2-9CEB-A465D8D3F0B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B79D86AF-463D-4824-9075-02786891185B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="46">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -62,14 +62,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>sortation_large_2000_3_errands.json</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>warehouse_large_5000.json</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>device=12400F, sim time = 5000</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -98,10 +90,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>卧槽，更新时代精神并没有更好的效果</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>instance</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -126,10 +114,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>比PIBT提升显著</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>PIBT mainstream update 30</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -158,14 +142,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>去掉没影响，可见不用担心任务饥饿的事情</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>融合后也没怎么变好，可见elapse确实没什么所谓</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>PIBT mainstream update 10</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -194,10 +170,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>hmm, 并没有比mainstream更好</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>compare_region_cos update 20</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -210,10 +182,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>region_cos比region_inner要好，但是不如PIBT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>PIBT anti-mainstream update 50</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -230,7 +198,15 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>反mainstream基本算不出来，可见逆潮流而动是不好的</t>
+    <t>不如update 20，可见切换太频繁也不好</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>去掉时间优先级就不行了，可见时间优先级的重要性</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>不如update 20，可见切换太慢是不好的</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -556,13 +532,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X28"/>
+  <dimension ref="A1:T28"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -570,22 +546,22 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" t="s">
-        <v>22</v>
-      </c>
       <c r="H1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I1" t="s">
         <v>3</v>
@@ -612,33 +588,21 @@
         <v>8</v>
       </c>
       <c r="Q1" t="s">
-        <v>2</v>
-      </c>
-      <c r="R1" t="s">
+        <v>1</v>
+      </c>
+      <c r="T1" t="s">
         <v>9</v>
       </c>
-      <c r="S1" t="s">
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="T1" t="s">
-        <v>2</v>
-      </c>
-      <c r="U1" t="s">
-        <v>1</v>
-      </c>
-      <c r="X1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E2">
         <v>100</v>
@@ -647,21 +611,21 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>3573</v>
+        <v>3534</v>
       </c>
       <c r="H2">
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E3">
         <v>150</v>
@@ -669,48 +633,42 @@
       <c r="F3">
         <v>1</v>
       </c>
-      <c r="G3">
-        <v>5635</v>
-      </c>
-      <c r="H3">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4">
+        <v>100</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>13</v>
       </c>
-      <c r="D4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4">
-        <v>100</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4" t="s">
-        <v>29</v>
-      </c>
-      <c r="H4" t="s">
-        <v>29</v>
-      </c>
-      <c r="U4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E5">
         <v>100</v>
@@ -719,21 +677,21 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>3505</v>
+        <v>3534</v>
       </c>
       <c r="H5">
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E6">
         <v>100</v>
@@ -741,25 +699,16 @@
       <c r="F6">
         <v>1</v>
       </c>
-      <c r="G6" t="s">
-        <v>29</v>
-      </c>
-      <c r="H6" t="s">
-        <v>29</v>
-      </c>
-      <c r="U6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E7">
         <v>150</v>
@@ -767,25 +716,16 @@
       <c r="F7">
         <v>1</v>
       </c>
-      <c r="G7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H7" t="s">
-        <v>29</v>
-      </c>
-      <c r="U7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E8">
         <v>150</v>
@@ -793,22 +733,16 @@
       <c r="F8">
         <v>2</v>
       </c>
-      <c r="G8" t="s">
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>29</v>
       </c>
-      <c r="H8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>35</v>
-      </c>
       <c r="C9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E9">
         <v>100</v>
@@ -817,21 +751,24 @@
         <v>1</v>
       </c>
       <c r="G9">
-        <v>3761</v>
+        <v>3804</v>
       </c>
       <c r="H9">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E10">
         <v>100</v>
@@ -840,21 +777,21 @@
         <v>1</v>
       </c>
       <c r="G10">
-        <v>3713</v>
+        <v>3638</v>
       </c>
       <c r="H10">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E11">
         <v>100</v>
@@ -863,21 +800,24 @@
         <v>1</v>
       </c>
       <c r="G11">
-        <v>3852</v>
+        <v>3975</v>
       </c>
       <c r="H11">
         <v>94</v>
       </c>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="Q11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E12">
         <v>100</v>
@@ -886,24 +826,24 @@
         <v>1</v>
       </c>
       <c r="G12">
-        <v>4195</v>
+        <v>4334</v>
       </c>
       <c r="H12">
-        <v>152</v>
-      </c>
-      <c r="U12" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+        <v>154</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D13" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E13">
         <v>100</v>
@@ -911,22 +851,16 @@
       <c r="F13">
         <v>1</v>
       </c>
-      <c r="G13" t="s">
-        <v>29</v>
-      </c>
-      <c r="H13" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E14">
         <v>100</v>
@@ -934,22 +868,16 @@
       <c r="F14">
         <v>1</v>
       </c>
-      <c r="G14" t="s">
-        <v>29</v>
-      </c>
-      <c r="H14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D15" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E15">
         <v>100</v>
@@ -957,22 +885,16 @@
       <c r="F15">
         <v>1</v>
       </c>
-      <c r="G15" t="s">
-        <v>29</v>
-      </c>
-      <c r="H15" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C16" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D16" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E16">
         <v>100</v>
@@ -980,311 +902,209 @@
       <c r="F16">
         <v>1</v>
       </c>
-      <c r="G16" t="s">
-        <v>29</v>
-      </c>
-      <c r="H16" t="s">
-        <v>29</v>
-      </c>
-      <c r="U16" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17">
+        <v>100</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18">
+        <v>100</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19">
+        <v>100</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" t="s">
+        <v>17</v>
+      </c>
+      <c r="E20">
+        <v>100</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" t="s">
+        <v>17</v>
+      </c>
+      <c r="E21">
+        <v>100</v>
+      </c>
+      <c r="F21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>30</v>
       </c>
-      <c r="C17" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" t="s">
-        <v>20</v>
-      </c>
-      <c r="E17">
-        <v>100</v>
-      </c>
-      <c r="F17">
-        <v>1</v>
-      </c>
-      <c r="G17">
-        <v>3781</v>
-      </c>
-      <c r="H17">
-        <v>75</v>
-      </c>
-      <c r="U17" t="s">
+      <c r="C22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22">
+        <v>100</v>
+      </c>
+      <c r="F22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" t="s">
+        <v>17</v>
+      </c>
+      <c r="E23">
+        <v>100</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>31</v>
-      </c>
-      <c r="C18" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" t="s">
-        <v>20</v>
-      </c>
-      <c r="E18">
-        <v>100</v>
-      </c>
-      <c r="F18">
-        <v>1</v>
-      </c>
-      <c r="G18">
-        <v>3772</v>
-      </c>
-      <c r="H18">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>32</v>
-      </c>
-      <c r="C19" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E19">
-        <v>100</v>
-      </c>
-      <c r="F19">
-        <v>1</v>
-      </c>
-      <c r="G19">
-        <v>3974</v>
-      </c>
-      <c r="H19">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="C24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24">
+        <v>100</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>35</v>
+      </c>
+      <c r="C25" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25">
+        <v>100</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>36</v>
+      </c>
+      <c r="C26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" t="s">
+        <v>17</v>
+      </c>
+      <c r="E26">
+        <v>100</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" t="s">
+        <v>17</v>
+      </c>
+      <c r="E27">
+        <v>100</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>38</v>
       </c>
-      <c r="C20" t="s">
-        <v>13</v>
-      </c>
-      <c r="D20" t="s">
-        <v>20</v>
-      </c>
-      <c r="E20">
-        <v>100</v>
-      </c>
-      <c r="F20">
-        <v>1</v>
-      </c>
-      <c r="G20" t="s">
-        <v>29</v>
-      </c>
-      <c r="H20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>37</v>
-      </c>
-      <c r="C21" t="s">
-        <v>13</v>
-      </c>
-      <c r="D21" t="s">
-        <v>20</v>
-      </c>
-      <c r="E21">
-        <v>100</v>
-      </c>
-      <c r="F21">
-        <v>1</v>
-      </c>
-      <c r="G21">
-        <v>3632</v>
-      </c>
-      <c r="H21">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>36</v>
-      </c>
-      <c r="C22" t="s">
-        <v>13</v>
-      </c>
-      <c r="D22" t="s">
-        <v>20</v>
-      </c>
-      <c r="E22">
-        <v>100</v>
-      </c>
-      <c r="F22">
-        <v>1</v>
-      </c>
-      <c r="G22">
-        <v>3877</v>
-      </c>
-      <c r="H22">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" t="s">
-        <v>20</v>
-      </c>
-      <c r="E23">
-        <v>100</v>
-      </c>
-      <c r="F23">
-        <v>1</v>
-      </c>
-      <c r="G23">
-        <v>3741</v>
-      </c>
-      <c r="H23">
-        <v>92</v>
-      </c>
-      <c r="U23" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>40</v>
-      </c>
-      <c r="C24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" t="s">
-        <v>20</v>
-      </c>
-      <c r="E24">
-        <v>100</v>
-      </c>
-      <c r="F24">
-        <v>1</v>
-      </c>
-      <c r="G24">
-        <v>4008</v>
-      </c>
-      <c r="H24">
-        <v>102</v>
-      </c>
-      <c r="U24" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>41</v>
-      </c>
-      <c r="C25" t="s">
-        <v>13</v>
-      </c>
-      <c r="D25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E25">
-        <v>100</v>
-      </c>
-      <c r="F25">
-        <v>1</v>
-      </c>
-      <c r="G25">
-        <v>3748</v>
-      </c>
-      <c r="H25">
-        <v>102</v>
-      </c>
-      <c r="U25" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" t="s">
-        <v>13</v>
-      </c>
-      <c r="D26" t="s">
-        <v>20</v>
-      </c>
-      <c r="E26">
-        <v>100</v>
-      </c>
-      <c r="F26">
-        <v>1</v>
-      </c>
-      <c r="G26">
-        <v>3592</v>
-      </c>
-      <c r="H26">
-        <v>73</v>
-      </c>
-      <c r="U26" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27" t="s">
-        <v>13</v>
-      </c>
-      <c r="D27" t="s">
-        <v>20</v>
-      </c>
-      <c r="E27">
-        <v>100</v>
-      </c>
-      <c r="F27">
-        <v>1</v>
-      </c>
-      <c r="G27">
-        <v>3679</v>
-      </c>
-      <c r="H27">
-        <v>75</v>
-      </c>
-      <c r="U27" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>45</v>
-      </c>
       <c r="C28" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E28">
         <v>100</v>
       </c>
       <c r="F28">
         <v>1</v>
-      </c>
-      <c r="G28">
-        <v>3885</v>
-      </c>
-      <c r="H28">
-        <v>86</v>
-      </c>
-      <c r="U28" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
std::sort(A.begin(), A.end(), compare_cos); // 按优先级排序
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B81A3DF4-69B6-4EBA-B845-48EF0B4FFFA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{791191FE-C6BE-4F0D-9C78-2ADA4C689E24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="53">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -231,6 +231,10 @@
   </si>
   <si>
     <t>把mainstream放在第二比较位</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>比对应的maintream update要好</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1125,6 +1129,15 @@
       <c r="F24">
         <v>1</v>
       </c>
+      <c r="G24">
+        <v>3567</v>
+      </c>
+      <c r="H24">
+        <v>76</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
@@ -1142,6 +1155,15 @@
       <c r="F25">
         <v>1</v>
       </c>
+      <c r="G25">
+        <v>3699</v>
+      </c>
+      <c r="H25">
+        <v>73</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
@@ -1158,6 +1180,15 @@
       </c>
       <c r="F26">
         <v>1</v>
+      </c>
+      <c r="G26">
+        <v>3928</v>
+      </c>
+      <c r="H26">
+        <v>77</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
std::sort(A.begin(), A.end(), compare_addition); // 按优先级排序
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EC2130F-FD35-46CA-B3B6-0D29B9D8028C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E82D20D-EA24-4E85-AC81-79A79F96E1D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1094,6 +1094,12 @@
       <c r="F21">
         <v>1</v>
       </c>
+      <c r="G21">
+        <v>3555</v>
+      </c>
+      <c r="H21">
+        <v>73</v>
+      </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
@@ -1111,6 +1117,12 @@
       <c r="F22">
         <v>1</v>
       </c>
+      <c r="G22">
+        <v>3800</v>
+      </c>
+      <c r="H22">
+        <v>82</v>
+      </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
@@ -1127,6 +1139,12 @@
       </c>
       <c r="F23">
         <v>1</v>
+      </c>
+      <c r="G23">
+        <v>4125</v>
+      </c>
+      <c r="H23">
+        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
std::sort(A.begin(), A.end(), compare_mainstream); // 按mainstream优先级排序
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D2C0597-A2CD-40BC-9CB4-9B235E1EB149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027A5F2C-1173-41D2-8FE1-291F4B009844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="71">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -295,6 +295,18 @@
   </si>
   <si>
     <t>2nd compare_region_cos update 50</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2nd mainstream update 20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2nd mainstream update 30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2nd mainstream update 50</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -620,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R44"/>
+  <dimension ref="A1:R47"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.08203125" customWidth="1"/>
@@ -1026,7 +1038,7 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="C17" t="s">
         <v>9</v>
@@ -1039,20 +1051,11 @@
       </c>
       <c r="F17">
         <v>1</v>
-      </c>
-      <c r="G17" t="s">
-        <v>23</v>
-      </c>
-      <c r="H17" t="s">
-        <v>23</v>
-      </c>
-      <c r="O17" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="C18" t="s">
         <v>9</v>
@@ -1065,20 +1068,11 @@
       </c>
       <c r="F18">
         <v>1</v>
-      </c>
-      <c r="G18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H18" t="s">
-        <v>23</v>
-      </c>
-      <c r="O18" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>38</v>
+        <v>70</v>
       </c>
       <c r="C19" t="s">
         <v>9</v>
@@ -1091,20 +1085,11 @@
       </c>
       <c r="F19">
         <v>1</v>
-      </c>
-      <c r="G19" t="s">
-        <v>23</v>
-      </c>
-      <c r="H19" t="s">
-        <v>23</v>
-      </c>
-      <c r="O19" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C20" t="s">
         <v>9</v>
@@ -1130,7 +1115,7 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="C21" t="s">
         <v>9</v>
@@ -1144,19 +1129,19 @@
       <c r="F21">
         <v>1</v>
       </c>
-      <c r="G21">
-        <v>3555</v>
-      </c>
-      <c r="H21">
-        <v>73</v>
+      <c r="G21" t="s">
+        <v>23</v>
+      </c>
+      <c r="H21" t="s">
+        <v>23</v>
       </c>
       <c r="O21" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="C22" t="s">
         <v>9</v>
@@ -1170,19 +1155,19 @@
       <c r="F22">
         <v>1</v>
       </c>
-      <c r="G22">
-        <v>3800</v>
-      </c>
-      <c r="H22">
-        <v>82</v>
+      <c r="G22" t="s">
+        <v>23</v>
+      </c>
+      <c r="H22" t="s">
+        <v>23</v>
       </c>
       <c r="O22" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="C23" t="s">
         <v>9</v>
@@ -1196,19 +1181,19 @@
       <c r="F23">
         <v>1</v>
       </c>
-      <c r="G23">
-        <v>4125</v>
-      </c>
-      <c r="H23">
-        <v>122</v>
+      <c r="G23" t="s">
+        <v>23</v>
+      </c>
+      <c r="H23" t="s">
+        <v>23</v>
       </c>
       <c r="O23" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="C24" t="s">
         <v>9</v>
@@ -1223,18 +1208,18 @@
         <v>1</v>
       </c>
       <c r="G24">
-        <v>3523</v>
+        <v>3555</v>
       </c>
       <c r="H24">
         <v>73</v>
       </c>
       <c r="O24" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="C25" t="s">
         <v>9</v>
@@ -1249,18 +1234,18 @@
         <v>1</v>
       </c>
       <c r="G25">
-        <v>3525</v>
+        <v>3800</v>
       </c>
       <c r="H25">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="O25" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="C26" t="s">
         <v>9</v>
@@ -1275,18 +1260,18 @@
         <v>1</v>
       </c>
       <c r="G26">
-        <v>3575</v>
+        <v>4125</v>
       </c>
       <c r="H26">
-        <v>73</v>
+        <v>122</v>
       </c>
       <c r="O26" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="C27" t="s">
         <v>9</v>
@@ -1301,18 +1286,18 @@
         <v>1</v>
       </c>
       <c r="G27">
-        <v>3567</v>
+        <v>3523</v>
       </c>
       <c r="H27">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="O27" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="C28" t="s">
         <v>9</v>
@@ -1327,18 +1312,18 @@
         <v>1</v>
       </c>
       <c r="G28">
-        <v>3699</v>
+        <v>3525</v>
       </c>
       <c r="H28">
         <v>73</v>
       </c>
       <c r="O28" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="C29" t="s">
         <v>9</v>
@@ -1353,18 +1338,18 @@
         <v>1</v>
       </c>
       <c r="G29">
-        <v>3928</v>
+        <v>3575</v>
       </c>
       <c r="H29">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="O29" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="C30" t="s">
         <v>9</v>
@@ -1379,18 +1364,18 @@
         <v>1</v>
       </c>
       <c r="G30">
-        <v>3503</v>
+        <v>3567</v>
       </c>
       <c r="H30">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O30" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="C31" t="s">
         <v>9</v>
@@ -1405,18 +1390,18 @@
         <v>1</v>
       </c>
       <c r="G31">
-        <v>3498</v>
+        <v>3699</v>
       </c>
       <c r="H31">
         <v>73</v>
       </c>
       <c r="O31" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="C32" t="s">
         <v>9</v>
@@ -1431,18 +1416,18 @@
         <v>1</v>
       </c>
       <c r="G32">
-        <v>3515</v>
+        <v>3928</v>
       </c>
       <c r="H32">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="O32" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="C33" t="s">
         <v>9</v>
@@ -1457,18 +1442,18 @@
         <v>1</v>
       </c>
       <c r="G33">
-        <v>3791</v>
+        <v>3503</v>
       </c>
       <c r="H33">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="O33" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="C34" t="s">
         <v>9</v>
@@ -1483,18 +1468,18 @@
         <v>1</v>
       </c>
       <c r="G34">
-        <v>4008</v>
+        <v>3498</v>
       </c>
       <c r="H34">
-        <v>102</v>
+        <v>73</v>
       </c>
       <c r="O34" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C35" t="s">
         <v>9</v>
@@ -1509,18 +1494,18 @@
         <v>1</v>
       </c>
       <c r="G35">
-        <v>3748</v>
+        <v>3515</v>
       </c>
       <c r="H35">
-        <v>102</v>
+        <v>73</v>
       </c>
       <c r="O35" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="C36" t="s">
         <v>9</v>
@@ -1535,18 +1520,18 @@
         <v>1</v>
       </c>
       <c r="G36">
-        <v>3584</v>
+        <v>3791</v>
       </c>
       <c r="H36">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="O36" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="C37" t="s">
         <v>9</v>
@@ -1561,18 +1546,18 @@
         <v>1</v>
       </c>
       <c r="G37">
-        <v>3538</v>
+        <v>4008</v>
       </c>
       <c r="H37">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="O37" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="C38" t="s">
         <v>9</v>
@@ -1587,18 +1572,18 @@
         <v>1</v>
       </c>
       <c r="G38">
-        <v>3576</v>
+        <v>3748</v>
       </c>
       <c r="H38">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="O38" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="C39" t="s">
         <v>9</v>
@@ -1613,7 +1598,7 @@
         <v>1</v>
       </c>
       <c r="G39">
-        <v>3632</v>
+        <v>3584</v>
       </c>
       <c r="H39">
         <v>73</v>
@@ -1624,7 +1609,7 @@
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="C40" t="s">
         <v>9</v>
@@ -1638,11 +1623,11 @@
       <c r="F40">
         <v>1</v>
       </c>
-      <c r="G40" t="s">
-        <v>23</v>
-      </c>
-      <c r="H40" t="s">
-        <v>23</v>
+      <c r="G40">
+        <v>3538</v>
+      </c>
+      <c r="H40">
+        <v>73</v>
       </c>
       <c r="O40" t="s">
         <v>64</v>
@@ -1650,7 +1635,7 @@
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="C41" t="s">
         <v>9</v>
@@ -1665,10 +1650,10 @@
         <v>1</v>
       </c>
       <c r="G41">
-        <v>3901</v>
+        <v>3576</v>
       </c>
       <c r="H41">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="O41" t="s">
         <v>64</v>
@@ -1676,7 +1661,7 @@
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="C42" t="s">
         <v>9</v>
@@ -1691,7 +1676,7 @@
         <v>1</v>
       </c>
       <c r="G42">
-        <v>3550</v>
+        <v>3632</v>
       </c>
       <c r="H42">
         <v>73</v>
@@ -1702,7 +1687,7 @@
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="C43" t="s">
         <v>9</v>
@@ -1716,39 +1701,117 @@
       <c r="F43">
         <v>1</v>
       </c>
-      <c r="G43">
-        <v>3517</v>
-      </c>
-      <c r="H43">
-        <v>73</v>
+      <c r="G43" t="s">
+        <v>23</v>
+      </c>
+      <c r="H43" t="s">
+        <v>23</v>
       </c>
       <c r="O43" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
+        <v>36</v>
+      </c>
+      <c r="C44" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" t="s">
+        <v>15</v>
+      </c>
+      <c r="E44">
+        <v>100</v>
+      </c>
+      <c r="F44">
+        <v>1</v>
+      </c>
+      <c r="G44">
+        <v>3901</v>
+      </c>
+      <c r="H44">
+        <v>87</v>
+      </c>
+      <c r="O44" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>65</v>
+      </c>
+      <c r="C45" t="s">
+        <v>9</v>
+      </c>
+      <c r="D45" t="s">
+        <v>15</v>
+      </c>
+      <c r="E45">
+        <v>100</v>
+      </c>
+      <c r="F45">
+        <v>1</v>
+      </c>
+      <c r="G45">
+        <v>3550</v>
+      </c>
+      <c r="H45">
+        <v>73</v>
+      </c>
+      <c r="O45" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>66</v>
+      </c>
+      <c r="C46" t="s">
+        <v>9</v>
+      </c>
+      <c r="D46" t="s">
+        <v>15</v>
+      </c>
+      <c r="E46">
+        <v>100</v>
+      </c>
+      <c r="F46">
+        <v>1</v>
+      </c>
+      <c r="G46">
+        <v>3517</v>
+      </c>
+      <c r="H46">
+        <v>73</v>
+      </c>
+      <c r="O46" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
         <v>67</v>
       </c>
-      <c r="C44" t="s">
-        <v>9</v>
-      </c>
-      <c r="D44" t="s">
-        <v>15</v>
-      </c>
-      <c r="E44">
-        <v>100</v>
-      </c>
-      <c r="F44">
-        <v>1</v>
-      </c>
-      <c r="G44">
+      <c r="C47" t="s">
+        <v>9</v>
+      </c>
+      <c r="D47" t="s">
+        <v>15</v>
+      </c>
+      <c r="E47">
+        <v>100</v>
+      </c>
+      <c r="F47">
+        <v>1</v>
+      </c>
+      <c r="G47">
         <v>3547</v>
       </c>
-      <c r="H44">
-        <v>73</v>
-      </c>
-      <c r="O44" t="s">
+      <c r="H47">
+        <v>73</v>
+      </c>
+      <c r="O47" t="s">
         <v>64</v>
       </c>
     </row>

</xml_diff>

<commit_message>
static bool compare_anti_cos(const Agent* a, const Agent* b)
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0E70EAD-5CD2-4949-B6A9-5270156A5462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB0F3E6-F2A4-4541-B83A-077BC613393D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="72">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -287,18 +287,6 @@
   </si>
   <si>
     <t>2nd compare_region_cos update 50</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2nd mainstream update 20</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2nd mainstream update 30</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2nd mainstream update 50</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -648,7 +636,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q50"/>
+  <dimension ref="A1:Q47"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.08203125" customWidth="1"/>
@@ -991,7 +979,7 @@
         <v>73</v>
       </c>
       <c r="N14" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
@@ -1017,7 +1005,7 @@
         <v>73</v>
       </c>
       <c r="N15" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
@@ -1051,7 +1039,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="C17" t="s">
         <v>9</v>
@@ -1064,11 +1052,20 @@
       </c>
       <c r="F17">
         <v>1</v>
+      </c>
+      <c r="G17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H17" t="s">
+        <v>23</v>
+      </c>
+      <c r="N17" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="C18" t="s">
         <v>9</v>
@@ -1081,11 +1078,20 @@
       </c>
       <c r="F18">
         <v>1</v>
+      </c>
+      <c r="G18" t="s">
+        <v>23</v>
+      </c>
+      <c r="H18" t="s">
+        <v>23</v>
+      </c>
+      <c r="N18" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="C19" t="s">
         <v>9</v>
@@ -1098,11 +1104,20 @@
       </c>
       <c r="F19">
         <v>1</v>
+      </c>
+      <c r="G19" t="s">
+        <v>23</v>
+      </c>
+      <c r="H19" t="s">
+        <v>23</v>
+      </c>
+      <c r="N19" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C20" t="s">
         <v>9</v>
@@ -1123,12 +1138,12 @@
         <v>23</v>
       </c>
       <c r="N20" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="C21" t="s">
         <v>9</v>
@@ -1142,19 +1157,19 @@
       <c r="F21">
         <v>1</v>
       </c>
-      <c r="G21" t="s">
-        <v>23</v>
-      </c>
-      <c r="H21" t="s">
-        <v>23</v>
+      <c r="G21">
+        <v>3472</v>
+      </c>
+      <c r="H21">
+        <v>73</v>
       </c>
       <c r="N21" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="C22" t="s">
         <v>9</v>
@@ -1168,19 +1183,19 @@
       <c r="F22">
         <v>1</v>
       </c>
-      <c r="G22" t="s">
-        <v>23</v>
-      </c>
-      <c r="H22" t="s">
-        <v>23</v>
+      <c r="G22">
+        <v>3516</v>
+      </c>
+      <c r="H22">
+        <v>73</v>
       </c>
       <c r="N22" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>68</v>
       </c>
       <c r="C23" t="s">
         <v>9</v>
@@ -1194,19 +1209,19 @@
       <c r="F23">
         <v>1</v>
       </c>
-      <c r="G23" t="s">
-        <v>23</v>
-      </c>
-      <c r="H23" t="s">
-        <v>23</v>
+      <c r="G23">
+        <v>3511</v>
+      </c>
+      <c r="H23">
+        <v>73</v>
       </c>
       <c r="N23" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>69</v>
+        <v>24</v>
       </c>
       <c r="C24" t="s">
         <v>9</v>
@@ -1221,18 +1236,18 @@
         <v>1</v>
       </c>
       <c r="G24">
-        <v>3472</v>
+        <v>3555</v>
       </c>
       <c r="H24">
         <v>73</v>
       </c>
       <c r="N24" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="C25" t="s">
         <v>9</v>
@@ -1247,18 +1262,18 @@
         <v>1</v>
       </c>
       <c r="G25">
-        <v>3516</v>
+        <v>3800</v>
       </c>
       <c r="H25">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="N25" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>71</v>
+        <v>26</v>
       </c>
       <c r="C26" t="s">
         <v>9</v>
@@ -1273,18 +1288,18 @@
         <v>1</v>
       </c>
       <c r="G26">
-        <v>3511</v>
+        <v>4125</v>
       </c>
       <c r="H26">
-        <v>73</v>
+        <v>122</v>
       </c>
       <c r="N26" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="C27" t="s">
         <v>9</v>
@@ -1299,18 +1314,18 @@
         <v>1</v>
       </c>
       <c r="G27">
-        <v>3555</v>
+        <v>3523</v>
       </c>
       <c r="H27">
         <v>73</v>
       </c>
       <c r="N27" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="C28" t="s">
         <v>9</v>
@@ -1325,18 +1340,18 @@
         <v>1</v>
       </c>
       <c r="G28">
-        <v>3800</v>
+        <v>3525</v>
       </c>
       <c r="H28">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="N28" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="C29" t="s">
         <v>9</v>
@@ -1351,18 +1366,18 @@
         <v>1</v>
       </c>
       <c r="G29">
-        <v>4125</v>
+        <v>3575</v>
       </c>
       <c r="H29">
-        <v>122</v>
+        <v>73</v>
       </c>
       <c r="N29" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="C30" t="s">
         <v>9</v>
@@ -1377,18 +1392,18 @@
         <v>1</v>
       </c>
       <c r="G30">
-        <v>3523</v>
+        <v>3567</v>
       </c>
       <c r="H30">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="N30" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="C31" t="s">
         <v>9</v>
@@ -1403,18 +1418,18 @@
         <v>1</v>
       </c>
       <c r="G31">
-        <v>3525</v>
+        <v>3699</v>
       </c>
       <c r="H31">
         <v>73</v>
       </c>
       <c r="N31" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="C32" t="s">
         <v>9</v>
@@ -1429,18 +1444,18 @@
         <v>1</v>
       </c>
       <c r="G32">
-        <v>3575</v>
+        <v>3928</v>
       </c>
       <c r="H32">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="N32" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C33" t="s">
         <v>9</v>
@@ -1455,18 +1470,18 @@
         <v>1</v>
       </c>
       <c r="G33">
-        <v>3567</v>
+        <v>3503</v>
       </c>
       <c r="H33">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="N33" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="C34" t="s">
         <v>9</v>
@@ -1481,18 +1496,18 @@
         <v>1</v>
       </c>
       <c r="G34">
-        <v>3699</v>
+        <v>3498</v>
       </c>
       <c r="H34">
         <v>73</v>
       </c>
       <c r="N34" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="C35" t="s">
         <v>9</v>
@@ -1507,18 +1522,18 @@
         <v>1</v>
       </c>
       <c r="G35">
-        <v>3928</v>
+        <v>3515</v>
       </c>
       <c r="H35">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="N35" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="C36" t="s">
         <v>9</v>
@@ -1533,18 +1548,18 @@
         <v>1</v>
       </c>
       <c r="G36">
-        <v>3503</v>
+        <v>3791</v>
       </c>
       <c r="H36">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="N36" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="C37" t="s">
         <v>9</v>
@@ -1559,18 +1574,18 @@
         <v>1</v>
       </c>
       <c r="G37">
-        <v>3498</v>
+        <v>4008</v>
       </c>
       <c r="H37">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="N37" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="C38" t="s">
         <v>9</v>
@@ -1585,18 +1600,18 @@
         <v>1</v>
       </c>
       <c r="G38">
-        <v>3515</v>
+        <v>3748</v>
       </c>
       <c r="H38">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="N38" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="C39" t="s">
         <v>9</v>
@@ -1611,18 +1626,18 @@
         <v>1</v>
       </c>
       <c r="G39">
-        <v>3791</v>
+        <v>3584</v>
       </c>
       <c r="H39">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="N39" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="C40" t="s">
         <v>9</v>
@@ -1637,18 +1652,18 @@
         <v>1</v>
       </c>
       <c r="G40">
-        <v>4008</v>
+        <v>3538</v>
       </c>
       <c r="H40">
-        <v>102</v>
+        <v>73</v>
       </c>
       <c r="N40" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="C41" t="s">
         <v>9</v>
@@ -1663,18 +1678,18 @@
         <v>1</v>
       </c>
       <c r="G41">
-        <v>3748</v>
+        <v>3576</v>
       </c>
       <c r="H41">
-        <v>102</v>
+        <v>73</v>
       </c>
       <c r="N41" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>59</v>
+        <v>34</v>
       </c>
       <c r="C42" t="s">
         <v>9</v>
@@ -1689,7 +1704,7 @@
         <v>1</v>
       </c>
       <c r="G42">
-        <v>3584</v>
+        <v>3632</v>
       </c>
       <c r="H42">
         <v>73</v>
@@ -1700,7 +1715,7 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="C43" t="s">
         <v>9</v>
@@ -1714,11 +1729,11 @@
       <c r="F43">
         <v>1</v>
       </c>
-      <c r="G43">
-        <v>3538</v>
-      </c>
-      <c r="H43">
-        <v>73</v>
+      <c r="G43" t="s">
+        <v>23</v>
+      </c>
+      <c r="H43" t="s">
+        <v>23</v>
       </c>
       <c r="N43" t="s">
         <v>62</v>
@@ -1726,7 +1741,7 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="C44" t="s">
         <v>9</v>
@@ -1741,10 +1756,10 @@
         <v>1</v>
       </c>
       <c r="G44">
-        <v>3576</v>
+        <v>3901</v>
       </c>
       <c r="H44">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="N44" t="s">
         <v>62</v>
@@ -1752,7 +1767,7 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="C45" t="s">
         <v>9</v>
@@ -1767,7 +1782,7 @@
         <v>1</v>
       </c>
       <c r="G45">
-        <v>3632</v>
+        <v>3550</v>
       </c>
       <c r="H45">
         <v>73</v>
@@ -1778,7 +1793,7 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="C46" t="s">
         <v>9</v>
@@ -1792,19 +1807,19 @@
       <c r="F46">
         <v>1</v>
       </c>
-      <c r="G46" t="s">
-        <v>23</v>
-      </c>
-      <c r="H46" t="s">
-        <v>23</v>
+      <c r="G46">
+        <v>3517</v>
+      </c>
+      <c r="H46">
+        <v>73</v>
       </c>
       <c r="N46" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="C47" t="s">
         <v>9</v>
@@ -1819,90 +1834,12 @@
         <v>1</v>
       </c>
       <c r="G47">
-        <v>3901</v>
+        <v>3547</v>
       </c>
       <c r="H47">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="N47" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>63</v>
-      </c>
-      <c r="C48" t="s">
-        <v>9</v>
-      </c>
-      <c r="D48" t="s">
-        <v>15</v>
-      </c>
-      <c r="E48">
-        <v>100</v>
-      </c>
-      <c r="F48">
-        <v>1</v>
-      </c>
-      <c r="G48">
-        <v>3550</v>
-      </c>
-      <c r="H48">
-        <v>73</v>
-      </c>
-      <c r="N48" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>64</v>
-      </c>
-      <c r="C49" t="s">
-        <v>9</v>
-      </c>
-      <c r="D49" t="s">
-        <v>15</v>
-      </c>
-      <c r="E49">
-        <v>100</v>
-      </c>
-      <c r="F49">
-        <v>1</v>
-      </c>
-      <c r="G49">
-        <v>3517</v>
-      </c>
-      <c r="H49">
-        <v>73</v>
-      </c>
-      <c r="N49" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>65</v>
-      </c>
-      <c r="C50" t="s">
-        <v>9</v>
-      </c>
-      <c r="D50" t="s">
-        <v>15</v>
-      </c>
-      <c r="E50">
-        <v>100</v>
-      </c>
-      <c r="F50">
-        <v>1</v>
-      </c>
-      <c r="G50">
-        <v>3547</v>
-      </c>
-      <c r="H50">
-        <v>73</v>
-      </c>
-      <c r="N50" t="s">
         <v>62</v>
       </c>
     </row>

</xml_diff>

<commit_message>
std::sort(A.begin(), A.end(), compare_anti_cos); // 按优先级排序
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB0F3E6-F2A4-4541-B83A-077BC613393D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A387C23-6BDB-4F80-ADFE-6EFB9503000F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="75">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -311,6 +311,18 @@
   </si>
   <si>
     <t>估计是把已经到达目标点的agent优先了，所以卡住</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>anti compare_cos update 20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>anti compare_cos update 30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>anti compare_cos update 50</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -636,7 +648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q47"/>
+  <dimension ref="A1:Q50"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.08203125" customWidth="1"/>
@@ -1533,7 +1545,7 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>31</v>
+        <v>72</v>
       </c>
       <c r="C36" t="s">
         <v>9</v>
@@ -1548,18 +1560,15 @@
         <v>1</v>
       </c>
       <c r="G36">
-        <v>3791</v>
+        <v>3473</v>
       </c>
       <c r="H36">
-        <v>86</v>
-      </c>
-      <c r="N36" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="C37" t="s">
         <v>9</v>
@@ -1574,18 +1583,15 @@
         <v>1</v>
       </c>
       <c r="G37">
-        <v>4008</v>
+        <v>3515</v>
       </c>
       <c r="H37">
-        <v>102</v>
-      </c>
-      <c r="N37" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="C38" t="s">
         <v>9</v>
@@ -1600,18 +1606,15 @@
         <v>1</v>
       </c>
       <c r="G38">
-        <v>3748</v>
+        <v>3505</v>
       </c>
       <c r="H38">
-        <v>102</v>
-      </c>
-      <c r="N38" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="C39" t="s">
         <v>9</v>
@@ -1626,18 +1629,18 @@
         <v>1</v>
       </c>
       <c r="G39">
-        <v>3584</v>
+        <v>3791</v>
       </c>
       <c r="H39">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="N39" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="C40" t="s">
         <v>9</v>
@@ -1652,18 +1655,18 @@
         <v>1</v>
       </c>
       <c r="G40">
-        <v>3538</v>
+        <v>4008</v>
       </c>
       <c r="H40">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="N40" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="C41" t="s">
         <v>9</v>
@@ -1678,18 +1681,18 @@
         <v>1</v>
       </c>
       <c r="G41">
-        <v>3576</v>
+        <v>3748</v>
       </c>
       <c r="H41">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="N41" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>34</v>
+        <v>59</v>
       </c>
       <c r="C42" t="s">
         <v>9</v>
@@ -1704,7 +1707,7 @@
         <v>1</v>
       </c>
       <c r="G42">
-        <v>3632</v>
+        <v>3584</v>
       </c>
       <c r="H42">
         <v>73</v>
@@ -1715,7 +1718,7 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="C43" t="s">
         <v>9</v>
@@ -1729,11 +1732,11 @@
       <c r="F43">
         <v>1</v>
       </c>
-      <c r="G43" t="s">
-        <v>23</v>
-      </c>
-      <c r="H43" t="s">
-        <v>23</v>
+      <c r="G43">
+        <v>3538</v>
+      </c>
+      <c r="H43">
+        <v>73</v>
       </c>
       <c r="N43" t="s">
         <v>62</v>
@@ -1741,7 +1744,7 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="C44" t="s">
         <v>9</v>
@@ -1756,10 +1759,10 @@
         <v>1</v>
       </c>
       <c r="G44">
-        <v>3901</v>
+        <v>3576</v>
       </c>
       <c r="H44">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="N44" t="s">
         <v>62</v>
@@ -1767,7 +1770,7 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="C45" t="s">
         <v>9</v>
@@ -1782,7 +1785,7 @@
         <v>1</v>
       </c>
       <c r="G45">
-        <v>3550</v>
+        <v>3632</v>
       </c>
       <c r="H45">
         <v>73</v>
@@ -1793,7 +1796,7 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="C46" t="s">
         <v>9</v>
@@ -1807,39 +1810,117 @@
       <c r="F46">
         <v>1</v>
       </c>
-      <c r="G46">
-        <v>3517</v>
-      </c>
-      <c r="H46">
-        <v>73</v>
+      <c r="G46" t="s">
+        <v>23</v>
+      </c>
+      <c r="H46" t="s">
+        <v>23</v>
       </c>
       <c r="N46" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
+        <v>36</v>
+      </c>
+      <c r="C47" t="s">
+        <v>9</v>
+      </c>
+      <c r="D47" t="s">
+        <v>15</v>
+      </c>
+      <c r="E47">
+        <v>100</v>
+      </c>
+      <c r="F47">
+        <v>1</v>
+      </c>
+      <c r="G47">
+        <v>3901</v>
+      </c>
+      <c r="H47">
+        <v>87</v>
+      </c>
+      <c r="N47" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>63</v>
+      </c>
+      <c r="C48" t="s">
+        <v>9</v>
+      </c>
+      <c r="D48" t="s">
+        <v>15</v>
+      </c>
+      <c r="E48">
+        <v>100</v>
+      </c>
+      <c r="F48">
+        <v>1</v>
+      </c>
+      <c r="G48">
+        <v>3550</v>
+      </c>
+      <c r="H48">
+        <v>73</v>
+      </c>
+      <c r="N48" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>64</v>
+      </c>
+      <c r="C49" t="s">
+        <v>9</v>
+      </c>
+      <c r="D49" t="s">
+        <v>15</v>
+      </c>
+      <c r="E49">
+        <v>100</v>
+      </c>
+      <c r="F49">
+        <v>1</v>
+      </c>
+      <c r="G49">
+        <v>3517</v>
+      </c>
+      <c r="H49">
+        <v>73</v>
+      </c>
+      <c r="N49" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
         <v>65</v>
       </c>
-      <c r="C47" t="s">
-        <v>9</v>
-      </c>
-      <c r="D47" t="s">
-        <v>15</v>
-      </c>
-      <c r="E47">
-        <v>100</v>
-      </c>
-      <c r="F47">
-        <v>1</v>
-      </c>
-      <c r="G47">
+      <c r="C50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D50" t="s">
+        <v>15</v>
+      </c>
+      <c r="E50">
+        <v>100</v>
+      </c>
+      <c r="F50">
+        <v>1</v>
+      </c>
+      <c r="G50">
         <v>3547</v>
       </c>
-      <c r="H47">
-        <v>73</v>
-      </c>
-      <c r="N47" t="s">
+      <c r="H50">
+        <v>73</v>
+      </c>
+      <c r="N50" t="s">
         <v>62</v>
       </c>
     </row>

</xml_diff>

<commit_message>
static bool compare_anti_region_inner(const Agent* a, const Agent* b)
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6618FE9-3EEE-42EB-A680-9FB8185E5123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62D893BB-903D-4F5C-B416-1A5F9B509071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="78">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -324,6 +324,18 @@
   </si>
   <si>
     <t>anti compare_cos update 50</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>anti compare_region_inner update 20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>anti compare_region_inner update 30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>anti compare_region_inner update 50</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -649,7 +661,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q50"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.08203125" customWidth="1"/>
@@ -1771,7 +1783,7 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="C45" t="s">
         <v>9</v>
@@ -1784,20 +1796,11 @@
       </c>
       <c r="F45">
         <v>1</v>
-      </c>
-      <c r="G45">
-        <v>3632</v>
-      </c>
-      <c r="H45">
-        <v>73</v>
-      </c>
-      <c r="N45" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="C46" t="s">
         <v>9</v>
@@ -1810,20 +1813,11 @@
       </c>
       <c r="F46">
         <v>1</v>
-      </c>
-      <c r="G46" t="s">
-        <v>23</v>
-      </c>
-      <c r="H46" t="s">
-        <v>23</v>
-      </c>
-      <c r="N46" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>36</v>
+        <v>77</v>
       </c>
       <c r="C47" t="s">
         <v>9</v>
@@ -1836,20 +1830,11 @@
       </c>
       <c r="F47">
         <v>1</v>
-      </c>
-      <c r="G47">
-        <v>3901</v>
-      </c>
-      <c r="H47">
-        <v>87</v>
-      </c>
-      <c r="N47" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="C48" t="s">
         <v>9</v>
@@ -1864,7 +1849,7 @@
         <v>1</v>
       </c>
       <c r="G48">
-        <v>3550</v>
+        <v>3632</v>
       </c>
       <c r="H48">
         <v>73</v>
@@ -1875,7 +1860,7 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="C49" t="s">
         <v>9</v>
@@ -1889,39 +1874,117 @@
       <c r="F49">
         <v>1</v>
       </c>
-      <c r="G49">
-        <v>3517</v>
-      </c>
-      <c r="H49">
-        <v>73</v>
+      <c r="G49" t="s">
+        <v>23</v>
+      </c>
+      <c r="H49" t="s">
+        <v>23</v>
       </c>
       <c r="N49" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
+        <v>36</v>
+      </c>
+      <c r="C50" t="s">
+        <v>9</v>
+      </c>
+      <c r="D50" t="s">
+        <v>15</v>
+      </c>
+      <c r="E50">
+        <v>100</v>
+      </c>
+      <c r="F50">
+        <v>1</v>
+      </c>
+      <c r="G50">
+        <v>3901</v>
+      </c>
+      <c r="H50">
+        <v>87</v>
+      </c>
+      <c r="N50" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>63</v>
+      </c>
+      <c r="C51" t="s">
+        <v>9</v>
+      </c>
+      <c r="D51" t="s">
+        <v>15</v>
+      </c>
+      <c r="E51">
+        <v>100</v>
+      </c>
+      <c r="F51">
+        <v>1</v>
+      </c>
+      <c r="G51">
+        <v>3550</v>
+      </c>
+      <c r="H51">
+        <v>73</v>
+      </c>
+      <c r="N51" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>64</v>
+      </c>
+      <c r="C52" t="s">
+        <v>9</v>
+      </c>
+      <c r="D52" t="s">
+        <v>15</v>
+      </c>
+      <c r="E52">
+        <v>100</v>
+      </c>
+      <c r="F52">
+        <v>1</v>
+      </c>
+      <c r="G52">
+        <v>3517</v>
+      </c>
+      <c r="H52">
+        <v>73</v>
+      </c>
+      <c r="N52" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
         <v>65</v>
       </c>
-      <c r="C50" t="s">
-        <v>9</v>
-      </c>
-      <c r="D50" t="s">
-        <v>15</v>
-      </c>
-      <c r="E50">
-        <v>100</v>
-      </c>
-      <c r="F50">
-        <v>1</v>
-      </c>
-      <c r="G50">
+      <c r="C53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D53" t="s">
+        <v>15</v>
+      </c>
+      <c r="E53">
+        <v>100</v>
+      </c>
+      <c r="F53">
+        <v>1</v>
+      </c>
+      <c r="G53">
         <v>3547</v>
       </c>
-      <c r="H50">
-        <v>73</v>
-      </c>
-      <c r="N50" t="s">
+      <c r="H53">
+        <v>73</v>
+      </c>
+      <c r="N53" t="s">
         <v>62</v>
       </c>
     </row>

</xml_diff>

<commit_message>
std::sort(A.begin(), A.end(), compare_anti_region_inner); // 按优先级排序
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62D893BB-903D-4F5C-B416-1A5F9B509071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21CCF659-D2C0-4760-AF90-DD4363735A2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="79">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -336,6 +336,10 @@
   </si>
   <si>
     <t>anti compare_region_inner update 50</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>超过baseline</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1797,6 +1801,15 @@
       <c r="F45">
         <v>1</v>
       </c>
+      <c r="G45">
+        <v>3528</v>
+      </c>
+      <c r="H45">
+        <v>73</v>
+      </c>
+      <c r="N45" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
@@ -1814,6 +1827,15 @@
       <c r="F46">
         <v>1</v>
       </c>
+      <c r="G46">
+        <v>3545</v>
+      </c>
+      <c r="H46">
+        <v>73</v>
+      </c>
+      <c r="N46" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
@@ -1830,6 +1852,15 @@
       </c>
       <c r="F47">
         <v>1</v>
+      </c>
+      <c r="G47">
+        <v>3559</v>
+      </c>
+      <c r="H47">
+        <v>73</v>
+      </c>
+      <c r="N47" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
static bool compare_anti_region_cos(const Agent* a, const Agent* b)
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21CCF659-D2C0-4760-AF90-DD4363735A2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76423A52-71BE-491F-AB0A-0A9DD0DCBC41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="82">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -340,6 +340,18 @@
   </si>
   <si>
     <t>超过baseline</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>anti compare_region_cos update 20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>anti compare_region_cos update 30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>anti compare_region_cos update 50</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -665,7 +677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q53"/>
+  <dimension ref="A1:Q56"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.08203125" customWidth="1"/>
@@ -2017,6 +2029,57 @@
       </c>
       <c r="N53" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>79</v>
+      </c>
+      <c r="C54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D54" t="s">
+        <v>15</v>
+      </c>
+      <c r="E54">
+        <v>100</v>
+      </c>
+      <c r="F54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>80</v>
+      </c>
+      <c r="C55" t="s">
+        <v>9</v>
+      </c>
+      <c r="D55" t="s">
+        <v>15</v>
+      </c>
+      <c r="E55">
+        <v>100</v>
+      </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>81</v>
+      </c>
+      <c r="C56" t="s">
+        <v>9</v>
+      </c>
+      <c r="D56" t="s">
+        <v>15</v>
+      </c>
+      <c r="E56">
+        <v>100</v>
+      </c>
+      <c r="F56">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
std::sort(A.begin(), A.end(), compare_anti_region_cos); // 按优先级排序
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76423A52-71BE-491F-AB0A-0A9DD0DCBC41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9039E3C-4EDA-4143-ABAE-FC507DE48B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="83">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -352,6 +352,10 @@
   </si>
   <si>
     <t>anti compare_region_cos update 50</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>不如baseline，看来小算例区域分割并不好</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2047,6 +2051,15 @@
       <c r="F54">
         <v>1</v>
       </c>
+      <c r="G54">
+        <v>3581</v>
+      </c>
+      <c r="H54">
+        <v>73</v>
+      </c>
+      <c r="N54" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
@@ -2064,6 +2077,15 @@
       <c r="F55">
         <v>1</v>
       </c>
+      <c r="G55">
+        <v>3594</v>
+      </c>
+      <c r="H55">
+        <v>73</v>
+      </c>
+      <c r="N55" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
@@ -2080,6 +2102,15 @@
       </c>
       <c r="F56">
         <v>1</v>
+      </c>
+      <c r="G56">
+        <v>3551</v>
+      </c>
+      <c r="H56">
+        <v>73</v>
+      </c>
+      <c r="N56" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
if(timestep % 8 < 3)
</commit_message>
<xml_diff>
--- a/doc/PIBT-result.xlsx
+++ b/doc/PIBT-result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitcloud\pibt2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA27BF84-CC1B-4E6B-B4DF-96B7EECBFE3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6784FB21-E86E-46CE-B2ED-7C0B10ED16AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="89">
   <si>
     <t>solver</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -368,6 +368,18 @@
   </si>
   <si>
     <t>mainsteam 2 : anti 4 update 20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>mainsteam 3 : anti 5 update 20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>mainsteam 3 : anti 5 update 30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>mainsteam 3 : anti 5 update 50</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -693,7 +705,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q59"/>
+  <dimension ref="A1:Q62"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.08203125" customWidth="1"/>
@@ -1347,7 +1359,7 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>24</v>
+        <v>86</v>
       </c>
       <c r="C27" t="s">
         <v>9</v>
@@ -1360,20 +1372,11 @@
       </c>
       <c r="F27">
         <v>1</v>
-      </c>
-      <c r="G27">
-        <v>3555</v>
-      </c>
-      <c r="H27">
-        <v>73</v>
-      </c>
-      <c r="N27" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>25</v>
+        <v>87</v>
       </c>
       <c r="C28" t="s">
         <v>9</v>
@@ -1386,20 +1389,11 @@
       </c>
       <c r="F28">
         <v>1</v>
-      </c>
-      <c r="G28">
-        <v>3800</v>
-      </c>
-      <c r="H28">
-        <v>82</v>
-      </c>
-      <c r="N28" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>26</v>
+        <v>88</v>
       </c>
       <c r="C29" t="s">
         <v>9</v>
@@ -1412,20 +1406,11 @@
       </c>
       <c r="F29">
         <v>1</v>
-      </c>
-      <c r="G29">
-        <v>4125</v>
-      </c>
-      <c r="H29">
-        <v>122</v>
-      </c>
-      <c r="N29" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="C30" t="s">
         <v>9</v>
@@ -1440,18 +1425,18 @@
         <v>1</v>
       </c>
       <c r="G30">
-        <v>3523</v>
+        <v>3555</v>
       </c>
       <c r="H30">
         <v>73</v>
       </c>
       <c r="N30" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="C31" t="s">
         <v>9</v>
@@ -1466,18 +1451,18 @@
         <v>1</v>
       </c>
       <c r="G31">
-        <v>3525</v>
+        <v>3800</v>
       </c>
       <c r="H31">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="N31" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="C32" t="s">
         <v>9</v>
@@ -1492,18 +1477,18 @@
         <v>1</v>
       </c>
       <c r="G32">
-        <v>3575</v>
+        <v>4125</v>
       </c>
       <c r="H32">
-        <v>73</v>
+        <v>122</v>
       </c>
       <c r="N32" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="C33" t="s">
         <v>9</v>
@@ -1518,18 +1503,18 @@
         <v>1</v>
       </c>
       <c r="G33">
-        <v>3567</v>
+        <v>3523</v>
       </c>
       <c r="H33">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="N33" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="C34" t="s">
         <v>9</v>
@@ -1544,18 +1529,18 @@
         <v>1</v>
       </c>
       <c r="G34">
-        <v>3699</v>
+        <v>3525</v>
       </c>
       <c r="H34">
         <v>73</v>
       </c>
       <c r="N34" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="C35" t="s">
         <v>9</v>
@@ -1570,18 +1555,18 @@
         <v>1</v>
       </c>
       <c r="G35">
-        <v>3928</v>
+        <v>3575</v>
       </c>
       <c r="H35">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="N35" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="C36" t="s">
         <v>9</v>
@@ -1596,18 +1581,18 @@
         <v>1</v>
       </c>
       <c r="G36">
-        <v>3503</v>
+        <v>3567</v>
       </c>
       <c r="H36">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="N36" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="C37" t="s">
         <v>9</v>
@@ -1622,18 +1607,18 @@
         <v>1</v>
       </c>
       <c r="G37">
-        <v>3498</v>
+        <v>3699</v>
       </c>
       <c r="H37">
         <v>73</v>
       </c>
       <c r="N37" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="C38" t="s">
         <v>9</v>
@@ -1648,18 +1633,18 @@
         <v>1</v>
       </c>
       <c r="G38">
-        <v>3515</v>
+        <v>3928</v>
       </c>
       <c r="H38">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="N38" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="C39" t="s">
         <v>9</v>
@@ -1674,15 +1659,18 @@
         <v>1</v>
       </c>
       <c r="G39">
-        <v>3473</v>
+        <v>3503</v>
       </c>
       <c r="H39">
         <v>73</v>
+      </c>
+      <c r="N39" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="C40" t="s">
         <v>9</v>
@@ -1697,15 +1685,18 @@
         <v>1</v>
       </c>
       <c r="G40">
-        <v>3515</v>
+        <v>3498</v>
       </c>
       <c r="H40">
         <v>73</v>
+      </c>
+      <c r="N40" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>74</v>
+        <v>52</v>
       </c>
       <c r="C41" t="s">
         <v>9</v>
@@ -1720,15 +1711,18 @@
         <v>1</v>
       </c>
       <c r="G41">
-        <v>3505</v>
+        <v>3515</v>
       </c>
       <c r="H41">
         <v>73</v>
+      </c>
+      <c r="N41" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>31</v>
+        <v>72</v>
       </c>
       <c r="C42" t="s">
         <v>9</v>
@@ -1743,18 +1737,15 @@
         <v>1</v>
       </c>
       <c r="G42">
-        <v>3791</v>
+        <v>3473</v>
       </c>
       <c r="H42">
-        <v>86</v>
-      </c>
-      <c r="N42" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="C43" t="s">
         <v>9</v>
@@ -1769,18 +1760,15 @@
         <v>1</v>
       </c>
       <c r="G43">
-        <v>4008</v>
+        <v>3515</v>
       </c>
       <c r="H43">
-        <v>102</v>
-      </c>
-      <c r="N43" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="C44" t="s">
         <v>9</v>
@@ -1795,18 +1783,15 @@
         <v>1</v>
       </c>
       <c r="G44">
-        <v>3748</v>
+        <v>3505</v>
       </c>
       <c r="H44">
-        <v>102</v>
-      </c>
-      <c r="N44" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="C45" t="s">
         <v>9</v>
@@ -1821,18 +1806,18 @@
         <v>1</v>
       </c>
       <c r="G45">
-        <v>3584</v>
+        <v>3791</v>
       </c>
       <c r="H45">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="N45" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="C46" t="s">
         <v>9</v>
@@ -1847,18 +1832,18 @@
         <v>1</v>
       </c>
       <c r="G46">
-        <v>3538</v>
+        <v>4008</v>
       </c>
       <c r="H46">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="N46" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="C47" t="s">
         <v>9</v>
@@ -1873,18 +1858,18 @@
         <v>1</v>
       </c>
       <c r="G47">
-        <v>3576</v>
+        <v>3748</v>
       </c>
       <c r="H47">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="N47" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="C48" t="s">
         <v>9</v>
@@ -1899,18 +1884,18 @@
         <v>1</v>
       </c>
       <c r="G48">
-        <v>3528</v>
+        <v>3584</v>
       </c>
       <c r="H48">
         <v>73</v>
       </c>
       <c r="N48" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="C49" t="s">
         <v>9</v>
@@ -1925,7 +1910,7 @@
         <v>1</v>
       </c>
       <c r="G49">
-        <v>3545</v>
+        <v>3538</v>
       </c>
       <c r="H49">
         <v>73</v>
@@ -1936,7 +1921,7 @@
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="C50" t="s">
         <v>9</v>
@@ -1951,7 +1936,7 @@
         <v>1</v>
       </c>
       <c r="G50">
-        <v>3559</v>
+        <v>3576</v>
       </c>
       <c r="H50">
         <v>73</v>
@@ -1962,7 +1947,7 @@
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="C51" t="s">
         <v>9</v>
@@ -1977,18 +1962,18 @@
         <v>1</v>
       </c>
       <c r="G51">
-        <v>3632</v>
+        <v>3528</v>
       </c>
       <c r="H51">
         <v>73</v>
       </c>
       <c r="N51" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="C52" t="s">
         <v>9</v>
@@ -2002,11 +1987,11 @@
       <c r="F52">
         <v>1</v>
       </c>
-      <c r="G52" t="s">
-        <v>23</v>
-      </c>
-      <c r="H52" t="s">
-        <v>23</v>
+      <c r="G52">
+        <v>3545</v>
+      </c>
+      <c r="H52">
+        <v>73</v>
       </c>
       <c r="N52" t="s">
         <v>62</v>
@@ -2014,7 +1999,7 @@
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>36</v>
+        <v>77</v>
       </c>
       <c r="C53" t="s">
         <v>9</v>
@@ -2029,10 +2014,10 @@
         <v>1</v>
       </c>
       <c r="G53">
-        <v>3901</v>
+        <v>3559</v>
       </c>
       <c r="H53">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="N53" t="s">
         <v>62</v>
@@ -2040,7 +2025,7 @@
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="C54" t="s">
         <v>9</v>
@@ -2055,7 +2040,7 @@
         <v>1</v>
       </c>
       <c r="G54">
-        <v>3550</v>
+        <v>3632</v>
       </c>
       <c r="H54">
         <v>73</v>
@@ -2066,7 +2051,7 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="C55" t="s">
         <v>9</v>
@@ -2080,19 +2065,19 @@
       <c r="F55">
         <v>1</v>
       </c>
-      <c r="G55">
-        <v>3517</v>
-      </c>
-      <c r="H55">
-        <v>73</v>
+      <c r="G55" t="s">
+        <v>23</v>
+      </c>
+      <c r="H55" t="s">
+        <v>23</v>
       </c>
       <c r="N55" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="C56" t="s">
         <v>9</v>
@@ -2107,10 +2092,10 @@
         <v>1</v>
       </c>
       <c r="G56">
-        <v>3547</v>
+        <v>3901</v>
       </c>
       <c r="H56">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="N56" t="s">
         <v>62</v>
@@ -2118,7 +2103,7 @@
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C57" t="s">
         <v>9</v>
@@ -2133,18 +2118,18 @@
         <v>1</v>
       </c>
       <c r="G57">
-        <v>3581</v>
+        <v>3550</v>
       </c>
       <c r="H57">
         <v>73</v>
       </c>
       <c r="N57" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="C58" t="s">
         <v>9</v>
@@ -2159,38 +2144,116 @@
         <v>1</v>
       </c>
       <c r="G58">
-        <v>3594</v>
+        <v>3517</v>
       </c>
       <c r="H58">
         <v>73</v>
       </c>
       <c r="N58" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
+        <v>65</v>
+      </c>
+      <c r="C59" t="s">
+        <v>9</v>
+      </c>
+      <c r="D59" t="s">
+        <v>15</v>
+      </c>
+      <c r="E59">
+        <v>100</v>
+      </c>
+      <c r="F59">
+        <v>1</v>
+      </c>
+      <c r="G59">
+        <v>3547</v>
+      </c>
+      <c r="H59">
+        <v>73</v>
+      </c>
+      <c r="N59" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>79</v>
+      </c>
+      <c r="C60" t="s">
+        <v>9</v>
+      </c>
+      <c r="D60" t="s">
+        <v>15</v>
+      </c>
+      <c r="E60">
+        <v>100</v>
+      </c>
+      <c r="F60">
+        <v>1</v>
+      </c>
+      <c r="G60">
+        <v>3581</v>
+      </c>
+      <c r="H60">
+        <v>73</v>
+      </c>
+      <c r="N60" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>80</v>
+      </c>
+      <c r="C61" t="s">
+        <v>9</v>
+      </c>
+      <c r="D61" t="s">
+        <v>15</v>
+      </c>
+      <c r="E61">
+        <v>100</v>
+      </c>
+      <c r="F61">
+        <v>1</v>
+      </c>
+      <c r="G61">
+        <v>3594</v>
+      </c>
+      <c r="H61">
+        <v>73</v>
+      </c>
+      <c r="N61" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
         <v>81</v>
       </c>
-      <c r="C59" t="s">
-        <v>9</v>
-      </c>
-      <c r="D59" t="s">
-        <v>15</v>
-      </c>
-      <c r="E59">
-        <v>100</v>
-      </c>
-      <c r="F59">
-        <v>1</v>
-      </c>
-      <c r="G59">
+      <c r="C62" t="s">
+        <v>9</v>
+      </c>
+      <c r="D62" t="s">
+        <v>15</v>
+      </c>
+      <c r="E62">
+        <v>100</v>
+      </c>
+      <c r="F62">
+        <v>1</v>
+      </c>
+      <c r="G62">
         <v>3551</v>
       </c>
-      <c r="H59">
-        <v>73</v>
-      </c>
-      <c r="N59" t="s">
+      <c r="H62">
+        <v>73</v>
+      </c>
+      <c r="N62" t="s">
         <v>82</v>
       </c>
     </row>

</xml_diff>